<commit_message>
Catching up the grades.
</commit_message>
<xml_diff>
--- a/problem_sets/ps3_preliminary_grades.xlsx
+++ b/problem_sets/ps3_preliminary_grades.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grading Audit" sheetId="1" r:id="Rd5c23770ea4a4401"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preliminary Grades" sheetId="2" r:id="R88cc4761958640fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grading Audit" sheetId="1" r:id="R105d134bcde34780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preliminary Grades" sheetId="2" r:id="Rce6eebc8e8994946"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PS3UpdatedAuditTable" displayName="PS3UpdatedAuditTable" ref="A4:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PS3CurrentAuditTable" displayName="PS3CurrentAuditTable" ref="A4:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Last Name"/>
     <x:tableColumn id="2" name="Student ID"/>
@@ -171,7 +171,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PS3UpdatedGradesTable" displayName="PS3UpdatedGradesTable" ref="A1:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PS3CurrentGradesTable" displayName="PS3CurrentGradesTable" ref="A1:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Last Name"/>
     <x:tableColumn id="2" name="Student ID"/>
@@ -383,17 +383,17 @@
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="72" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Problem Set 3 Regraded — Updated Submissions</x:v>
+        <x:v>Problem Set 3 Regrade — Current Resubmissions</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="10" t="str">
-        <x:v>Rubric: Completeness, Bug-Free Execution, and Meets Requirements are equally weighted. Preliminary Grade = rounded mean of the three category scores. Earlier scores were preserved for unchanged submissions; new/current submissions were checked against the same Problem Set 3 requirements.</x:v>
+        <x:v>Rubric: Completeness, Bug-Free Execution, and Meets Requirements are equally weighted. Preliminary Grade = rounded mean of the three category scores. Current resubmitted material was re-evaluated; unchanged submissions retain the prior audit scores under the same rubric.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -578,7 +578,7 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="G10" s="27" t="str">
-        <x:v>New submission. Exercise 1 evaluates the requested values but omits the written pole explanations. In placement(), score 2 is excluded from the Trigonometry range, so Sophia is omitted from all rosters. Exercise 3 begins with i=1 and counts only later course records, producing Total: 3 rather than 6. The file executes without a Python runtime error, but the logic does not meet several stated requirements.</x:v>
+        <x:v>Exercise 1 evaluates the requested values but omits the written pole explanations. In placement(), score 2 is excluded from the Trigonometry range, so Sophia is omitted from all rosters. Exercise 3 begins with i=1 and counts only later course records, producing Total: 3 rather than 6. The file executes without a Python runtime error, but the logic does not meet several stated requirements.</x:v>
       </x:c>
       <x:c r="H10" s="27" t="str">
         <x:v>homework_3.py</x:v>
@@ -592,23 +592,23 @@
         <x:v>20693757</x:v>
       </x:c>
       <x:c r="C11" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D11" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E11" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="F11" s="26" t="n">
         <x:f>ROUND(AVERAGE(C11:E11),0)</x:f>
-        <x:v>0</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="G11" s="27" t="str">
-        <x:v>The submitted notebook contains Problem Set 2 work rather than Problem Set 3. It does not provide the required pole-function, placement-function, or roster-count exercises for Problem Set 3.</x:v>
+        <x:v>Resubmitted Problem Set 3 notebook now contains all three computational exercises and executes cleanly: the pole function is evaluated at the required values, placement() returns the correct courses, the required roster structure is built, and the while loop counts all six students. The remaining omissions are the requested written explanations for why x=1 is excluded, the magnitude/sign behavior near the pole, and why the final total should be 6.</x:v>
       </x:c>
       <x:c r="H11" s="27" t="str">
-        <x:v>Aleck_Lam_20693757_Problem_Set_3_Loops_and_Functions.ipynb</x:v>
+        <x:v>Copy of Aleck Lam 20693757 Problem Set 3 Loops and Functions .ipynb</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -713,7 +713,7 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="G15" s="27" t="str">
-        <x:v>New submission. Exercise 1 evaluates all requested values but omits the written pole explanations. Exercise 2 produces the correct rosters, although Trigonometry is misspelled internally and the requested placement tests for scores 1, 3, and 5 are omitted. Exercise 3 adds len(rosters[i]) instead of len(rosters[i][1]); it produces 6 only because each course record has two elements, and the final explanation is omitted.</x:v>
+        <x:v>Exercise 1 evaluates all requested values but omits the written pole explanations. Exercise 2 produces the correct rosters, although Trigonometry is misspelled internally and the requested placement tests for scores 1, 3, and 5 are omitted. Exercise 3 adds len(rosters[i]) instead of len(rosters[i][1]); it produces 6 only because each course record has two elements, and the final explanation is omitted.</x:v>
       </x:c>
       <x:c r="H15" s="27" t="str">
         <x:v>needles_20686013.ipynb</x:v>
@@ -902,7 +902,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="G22" s="27" t="str">
-        <x:v>New submission uploaded separately. All three exercises are complete and execute correctly: the pole function and explanations are present, placement() and the required roster structures are correct, and the single while loop counts all six students with an appropriate explanation.</x:v>
+        <x:v>All three exercises are complete and execute correctly: the pole function and explanations are present, placement() and the required roster structures are correct, and the single while loop counts all six students with an appropriate explanation.</x:v>
       </x:c>
       <x:c r="H22" s="27" t="str">
         <x:v>Problem_3__Tien_Dat_Tran.ipynb</x:v>
@@ -981,7 +981,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19963692d45c48cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26e765a2d8ff45c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1087,7 +1087,7 @@
       </x:c>
       <x:c r="C8" s="22" t="n">
         <x:f>'Grading Audit'!F11</x:f>
-        <x:v>0</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1261,7 +1261,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e554a2c56904486"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3b752aa0a414ddc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>